<commit_message>
Align MQTT schemas to REST and add comparison/rebuild tooling.
Sync MQTT split schemas and references to openAPISpec2.yaml, preserve MQTT path-param payload fields for certificates and userapps, and regenerate docs/openapi_md.json and RestAPI/FXR90-rest-api.yaml. Add compare, align, sync, and rebuild_and_verify scripts with a field alignment report showing 0 issues across 762 compared fields.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/RestAPI/schema_example_report.xlsx
+++ b/RestAPI/schema_example_report.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schema vs Example'!$A$1:$I$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schema vs Example'!$A$1:$I$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2798,7 +2798,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>/cloud/mode</t>
+          <t>/cloud/logs</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>/cloud/mode</t>
+          <t>/cloud/logs</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>set_mode_default_FXR90</t>
+          <t>set_logs</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
@@ -2881,15 +2881,19 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>request</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr"/>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -2897,7 +2901,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>set_mode_TAG_FOCUS</t>
+          <t>(inline example)</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
@@ -2913,7 +2917,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>/cloud/network</t>
+          <t>/cloud/mode</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -2934,7 +2938,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>set_Network_ethernet_dhcp</t>
+          <t>set_mode_default_FXR90</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
@@ -2950,7 +2954,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>/cloud/network</t>
+          <t>/cloud/mode</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -2971,7 +2975,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>set_Network_ethernet_dhcp_8021x_tls</t>
+          <t>set_mode_TAG_FOCUS</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
@@ -3008,7 +3012,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>set_Network_ethernet_dhcp_8021x_ttls_mschapv2</t>
+          <t>set_Network_ethernet_dhcp</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
@@ -3045,7 +3049,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>set_Network_ethernet_dhcp_8021x_peap_mschapv2</t>
+          <t>set_Network_ethernet_dhcp_8021x_tls</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
@@ -3082,7 +3086,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>set_Network_wifi_dhcp</t>
+          <t>set_Network_ethernet_dhcp_8021x_ttls_mschapv2</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
@@ -3119,7 +3123,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>set_Network_wifi_security_wpa2_personal</t>
+          <t>set_Network_ethernet_dhcp_8021x_peap_mschapv2</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
@@ -3156,7 +3160,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>set_Network_wifi_wpa2_enterprise_tls</t>
+          <t>set_Network_wifi_dhcp</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
@@ -3193,7 +3197,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>set_Network_wifi_wpa3_enterprise_ttls_mschapv2</t>
+          <t>set_Network_wifi_security_wpa2_personal</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
@@ -3230,7 +3234,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>set_Network_wifi_wpa2_enterprise_peap_tls</t>
+          <t>set_Network_wifi_wpa2_enterprise_tls</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
@@ -3267,7 +3271,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>set_Network_wifi_wpa2_enterprise_ttls_tls</t>
+          <t>set_Network_wifi_wpa3_enterprise_ttls_mschapv2</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
@@ -3304,7 +3308,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>set_Network_wifi_wpa3_enterprise_peap_mschapv2</t>
+          <t>set_Network_wifi_wpa2_enterprise_peap_tls</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
@@ -3341,7 +3345,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>set_Network_bluetooth</t>
+          <t>set_Network_wifi_wpa2_enterprise_ttls_tls</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
@@ -3378,7 +3382,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>set_Network_wan</t>
+          <t>set_Network_wifi_wpa3_enterprise_peap_mschapv2</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
@@ -3415,7 +3419,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>set_Network_hotspot</t>
+          <t>set_Network_bluetooth</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
@@ -3431,24 +3435,20 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>/cloud/networkInterfaces</t>
+          <t>/cloud/network</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>response</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -3456,7 +3456,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>application/json</t>
+          <t>set_Network_wan</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>/cloud/ntpServer</t>
+          <t>/cloud/network</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>set_ntpServer</t>
+          <t>set_Network_hotspot</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
@@ -3509,20 +3509,24 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>/cloud/ntpServer</t>
+          <t>/cloud/networkInterfaces</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>request</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr"/>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -3530,7 +3534,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>set_ntpServer_legacy</t>
+          <t>application/json</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
@@ -3546,7 +3550,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>/cloud/os</t>
+          <t>/cloud/ntpServer</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -3567,7 +3571,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>set_os</t>
+          <t>set_ntpServer</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
@@ -3583,7 +3587,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>/cloud/pass-through</t>
+          <t>/cloud/ntpServer</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -3604,7 +3608,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>set_passthru</t>
+          <t>set_ntpServer_legacy</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
@@ -3620,7 +3624,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>/cloud/pass-through</t>
+          <t>/cloud/os</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -3641,7 +3645,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>set_os</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
@@ -3657,7 +3661,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>/cloud/preSelection</t>
+          <t>/cloud/pass-through</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -3678,7 +3682,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>set_preSelection</t>
+          <t>set_passthru</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr">
@@ -3694,24 +3698,20 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>/cloud/readPoints</t>
+          <t>/cloud/pass-through</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>response</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>(inline example)</t>
+          <t>status</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
@@ -3735,24 +3735,20 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>/cloud/readerCapabilities</t>
+          <t>/cloud/preSelection</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>response</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -3760,7 +3756,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>(inline example)</t>
+          <t>set_preSelection</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
@@ -3776,7 +3772,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>/cloud/region</t>
+          <t>/cloud/readPoints</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -3801,7 +3797,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>multiple_values</t>
+          <t>(inline example)</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
@@ -3817,20 +3813,24 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>/cloud/region</t>
+          <t>/cloud/readerCapabilities</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>request</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr"/>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>set_region</t>
+          <t>(inline example)</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
@@ -3854,20 +3854,24 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>/cloud/revertbackOS</t>
+          <t>/cloud/region</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>request</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr"/>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -3875,7 +3879,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>set_revertbackOS</t>
+          <t>multiple_values</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
@@ -3891,7 +3895,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>/cloud/setdataToRG</t>
+          <t>/cloud/region</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -3912,7 +3916,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>set_dataToRG</t>
+          <t>set_region</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
@@ -3928,7 +3932,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>/cloud/stack-led</t>
+          <t>/cloud/revertbackOS</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -3949,7 +3953,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>red_high_alert</t>
+          <t>set_revertbackOS</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
@@ -3965,7 +3969,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>/cloud/stack-led</t>
+          <t>/cloud/setdataToRG</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -3986,7 +3990,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>green_solid</t>
+          <t>set_dataToRG</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
@@ -4002,7 +4006,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>/cloud/start</t>
+          <t>/cloud/stack-led</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -4023,7 +4027,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>start_Inventory</t>
+          <t>red_high_alert</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
@@ -4039,7 +4043,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>/cloud/start</t>
+          <t>/cloud/stack-led</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -4060,7 +4064,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>start_Inventory with AutoStart</t>
+          <t>green_solid</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr">
@@ -4097,7 +4101,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>start_Inventory with ImpinjGen2X</t>
+          <t>start_Inventory</t>
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr">
@@ -4134,7 +4138,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>start_BLE_only</t>
+          <t>start_Inventory with AutoStart</t>
         </is>
       </c>
       <c r="H96" s="4" t="inlineStr">
@@ -4171,7 +4175,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>start_RFID_only</t>
+          <t>start_Inventory with ImpinjGen2X</t>
         </is>
       </c>
       <c r="H97" s="4" t="inlineStr">
@@ -4208,7 +4212,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>start_BLE_and_RFID</t>
+          <t>start_BLE_only</t>
         </is>
       </c>
       <c r="H98" s="4" t="inlineStr">
@@ -4224,24 +4228,20 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>/cloud/status</t>
+          <t>/cloud/start</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>response</t>
-        </is>
-      </c>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr"/>
       <c r="F99" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>(inline example)</t>
+          <t>start_RFID_only</t>
         </is>
       </c>
       <c r="H99" s="4" t="inlineStr">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>/cloud/stop</t>
+          <t>/cloud/start</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>stop_RFID_default</t>
+          <t>start_BLE_and_RFID</t>
         </is>
       </c>
       <c r="H100" s="4" t="inlineStr">
@@ -4302,20 +4302,24 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>/cloud/stop</t>
+          <t>/cloud/status</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>request</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr"/>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -4323,7 +4327,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>stop_RFID_explicit</t>
+          <t>(inline example)</t>
         </is>
       </c>
       <c r="H101" s="4" t="inlineStr">
@@ -4360,7 +4364,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>stop_BLE_only</t>
+          <t>stop_RFID_default</t>
         </is>
       </c>
       <c r="H102" s="4" t="inlineStr">
@@ -4397,7 +4401,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>stop_BLE_and_RFID</t>
+          <t>stop_RFID_explicit</t>
         </is>
       </c>
       <c r="H103" s="4" t="inlineStr">
@@ -4413,24 +4417,20 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>/cloud/supportedRegionList</t>
+          <t>/cloud/stop</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>response</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr"/>
       <c r="F104" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -4438,7 +4438,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>(inline example)</t>
+          <t>stop_BLE_only</t>
         </is>
       </c>
       <c r="H104" s="4" t="inlineStr">
@@ -4454,24 +4454,20 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>/cloud/supportedStandardList</t>
+          <t>/cloud/stop</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>response</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr"/>
       <c r="F105" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -4479,7 +4475,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>(inline example)</t>
+          <t>stop_BLE_and_RFID</t>
         </is>
       </c>
       <c r="H105" s="4" t="inlineStr">
@@ -4495,20 +4491,24 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>/cloud/timeZone</t>
+          <t>/cloud/supportedRegionList</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>request</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr"/>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>set_timeZone</t>
+          <t>(inline example)</t>
         </is>
       </c>
       <c r="H106" s="4" t="inlineStr">
@@ -4532,20 +4532,24 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>/cloud/updatePassword</t>
+          <t>/cloud/supportedStandardList</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>request</t>
-        </is>
-      </c>
-      <c r="E107" s="2" t="inlineStr"/>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -4553,7 +4557,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>set_logs</t>
+          <t>(inline example)</t>
         </is>
       </c>
       <c r="H107" s="4" t="inlineStr">
@@ -4569,24 +4573,20 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>/cloud/version</t>
+          <t>/cloud/timeZone</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>response</t>
-        </is>
-      </c>
-      <c r="E108" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr"/>
       <c r="F108" s="2" t="inlineStr">
         <is>
           <t>application/json</t>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>(inline example)</t>
+          <t>set_timeZone</t>
         </is>
       </c>
       <c r="H108" s="4" t="inlineStr">
@@ -4610,43 +4610,121 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
+          <t>/cloud/updatePassword</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>request</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr"/>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>set_password</t>
+        </is>
+      </c>
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>/cloud/version</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>response</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>(inline example)</t>
+        </is>
+      </c>
+      <c r="H110" s="4" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
           <t>/cloud/wifiNetworks</t>
         </is>
       </c>
-      <c r="C109" s="2" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="D109" s="2" t="inlineStr">
+      <c r="D111" s="2" t="inlineStr">
         <is>
           <t>response</t>
         </is>
       </c>
-      <c r="E109" s="2" t="inlineStr">
+      <c r="E111" s="2" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t>application/json</t>
-        </is>
-      </c>
-      <c r="G109" s="2" t="inlineStr">
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>application/json</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
         <is>
           <t>(inline example)</t>
         </is>
       </c>
-      <c r="H109" s="4" t="inlineStr">
-        <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="I109" s="2" t="inlineStr"/>
+      <c r="H111" s="4" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I109"/>
+  <autoFilter ref="A1:I111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4681,7 +4759,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-08 16:04</t>
+          <t>Generated: 2026-07-08 21:32</t>
         </is>
       </c>
     </row>
@@ -4704,7 +4782,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7">
@@ -4724,7 +4802,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>